<commit_message>
Update results + New results
</commit_message>
<xml_diff>
--- a/Results/tables/Species_Density_and_Model_Coefficients_Summary.xlsx
+++ b/Results/tables/Species_Density_and_Model_Coefficients_Summary.xlsx
@@ -1062,43 +1062,43 @@
         </is>
       </c>
       <c r="C14">
-        <v>4.399524082903509</v>
+        <v>4.410839548191006</v>
       </c>
       <c r="D14">
-        <v>0.4515033947672068</v>
+        <v>0.467828769273879</v>
       </c>
       <c r="E14">
-        <v>0.01703103072752752</v>
+        <v>0.01130454264506064</v>
       </c>
       <c r="F14">
-        <v>4.369848808483351</v>
+        <v>4.373566168925842</v>
       </c>
       <c r="G14">
-        <v>3.619223080911201</v>
+        <v>3.596753068911467</v>
       </c>
       <c r="H14">
-        <v>3.725703299932598</v>
+        <v>3.707836193317775</v>
       </c>
       <c r="I14">
-        <v>3.856692583835749</v>
+        <v>3.845175006675777</v>
       </c>
       <c r="J14">
-        <v>4.084344492600104</v>
+        <v>4.084204196605862</v>
       </c>
       <c r="K14">
-        <v>4.369848808483351</v>
+        <v>4.373566168925842</v>
       </c>
       <c r="L14">
-        <v>4.66913632128504</v>
+        <v>4.696162248635995</v>
       </c>
       <c r="M14">
-        <v>4.978525010525605</v>
+        <v>5.033857068034441</v>
       </c>
       <c r="N14">
-        <v>5.198957201935871</v>
+        <v>5.24194276694994</v>
       </c>
       <c r="O14">
-        <v>5.392367958147705</v>
+        <v>5.430085206221917</v>
       </c>
     </row>
     <row r="15">
@@ -1113,43 +1113,43 @@
         </is>
       </c>
       <c r="C15">
-        <v>13246.96701362246</v>
+        <v>13281.03787960312</v>
       </c>
       <c r="D15">
-        <v>1359.47672164406</v>
+        <v>1408.63242428365</v>
       </c>
       <c r="E15">
-        <v>51.28043352058523</v>
+        <v>34.03797790427834</v>
       </c>
       <c r="F15">
-        <v>13157.61476234337</v>
+        <v>13168.80773463571</v>
       </c>
       <c r="G15">
-        <v>10897.48069662363</v>
+        <v>10829.82349049243</v>
       </c>
       <c r="H15">
-        <v>11218.09263609705</v>
+        <v>11164.29477807982</v>
       </c>
       <c r="I15">
-        <v>11612.50136992944</v>
+        <v>11577.82194510076</v>
       </c>
       <c r="J15">
-        <v>12297.96126721891</v>
+        <v>12297.53883598025</v>
       </c>
       <c r="K15">
-        <v>13157.61476234337</v>
+        <v>13168.80773463571</v>
       </c>
       <c r="L15">
-        <v>14058.76946338926</v>
+        <v>14140.14453064298</v>
       </c>
       <c r="M15">
-        <v>14990.33880669259</v>
+        <v>15156.9436318517</v>
       </c>
       <c r="N15">
-        <v>15654.06013502891</v>
+        <v>15783.48967128627</v>
       </c>
       <c r="O15">
-        <v>16236.41992198274</v>
+        <v>16349.98655593419</v>
       </c>
     </row>
     <row r="16">
@@ -1164,43 +1164,43 @@
         </is>
       </c>
       <c r="C16">
-        <v>4.678647967317327</v>
+        <v>4.690681332215209</v>
       </c>
       <c r="D16">
-        <v>0.4801486252509269</v>
+        <v>0.4975097485933698</v>
       </c>
       <c r="E16">
-        <v>0.01811154929332223</v>
+        <v>0.01202174927813127</v>
       </c>
       <c r="F16">
-        <v>4.647089971559334</v>
+        <v>4.651043176622045</v>
       </c>
       <c r="G16">
-        <v>3.848841463688045</v>
+        <v>3.824945861803132</v>
       </c>
       <c r="H16">
-        <v>3.962077225305965</v>
+        <v>3.943076556035821</v>
       </c>
       <c r="I16">
-        <v>4.101377007583637</v>
+        <v>4.089128708005659</v>
       </c>
       <c r="J16">
-        <v>4.343472088807363</v>
+        <v>4.343322891858802</v>
       </c>
       <c r="K16">
-        <v>4.647089971559334</v>
+        <v>4.651043176622045</v>
       </c>
       <c r="L16">
-        <v>4.965365513874121</v>
+        <v>4.994106077099305</v>
       </c>
       <c r="M16">
-        <v>5.294383092764388</v>
+        <v>5.353225643347804</v>
       </c>
       <c r="N16">
-        <v>5.528800408100988</v>
+        <v>5.574513153976976</v>
       </c>
       <c r="O16">
-        <v>5.734481937365534</v>
+        <v>5.774592122628746</v>
       </c>
     </row>
     <row r="17">
@@ -1215,43 +1215,43 @@
         </is>
       </c>
       <c r="C17">
-        <v>14087.40902959247</v>
+        <v>14123.64149129999</v>
       </c>
       <c r="D17">
-        <v>1445.727510630541</v>
+        <v>1498.001853014637</v>
       </c>
       <c r="E17">
-        <v>54.53387492219304</v>
+        <v>36.19748707645297</v>
       </c>
       <c r="F17">
-        <v>13992.38790436515</v>
+        <v>14004.29100480898</v>
       </c>
       <c r="G17">
-        <v>11588.8616471647</v>
+        <v>11516.91198988923</v>
       </c>
       <c r="H17">
-        <v>11929.81452539626</v>
+        <v>11872.60351022386</v>
       </c>
       <c r="I17">
-        <v>12349.24616983433</v>
+        <v>12312.36653980504</v>
       </c>
       <c r="J17">
-        <v>13078.19445939897</v>
+        <v>13077.74522738685</v>
       </c>
       <c r="K17">
-        <v>13992.38790436515</v>
+        <v>14004.29100480898</v>
       </c>
       <c r="L17">
-        <v>14950.71556227498</v>
+        <v>15037.25339814601</v>
       </c>
       <c r="M17">
-        <v>15941.38749231357</v>
+        <v>16118.56241212024</v>
       </c>
       <c r="N17">
-        <v>16647.21802879207</v>
+        <v>16784.85910662467</v>
       </c>
       <c r="O17">
-        <v>17266.52511340762</v>
+        <v>17387.29688123515</v>
       </c>
     </row>
     <row r="18">
@@ -4261,43 +4261,43 @@
         </is>
       </c>
       <c r="H40">
-        <v>0.5417060408592684</v>
+        <v>0.5336913927167031</v>
       </c>
       <c r="I40">
-        <v>0.2487964918880957</v>
+        <v>0.2519487102677469</v>
       </c>
       <c r="J40">
-        <v>0.02637162723743947</v>
+        <v>0.01807548370186413</v>
       </c>
       <c r="K40">
-        <v>0.5604503041457983</v>
+        <v>0.5420514501089884</v>
       </c>
       <c r="L40">
-        <v>-0.01666641103674497</v>
+        <v>0.01280902634430924</v>
       </c>
       <c r="M40">
-        <v>0.09536507547659817</v>
+        <v>0.1120212086109604</v>
       </c>
       <c r="N40">
-        <v>0.2182271469328651</v>
+        <v>0.2147962563771071</v>
       </c>
       <c r="O40">
-        <v>0.3848421882080577</v>
+        <v>0.3671732564636359</v>
       </c>
       <c r="P40">
-        <v>0.5604503041457983</v>
+        <v>0.5420514501089884</v>
       </c>
       <c r="Q40">
-        <v>0.716696337758487</v>
+        <v>0.7070879191567029</v>
       </c>
       <c r="R40">
-        <v>0.8442323233560615</v>
+        <v>0.8586412762319757</v>
       </c>
       <c r="S40">
-        <v>0.9268458555843748</v>
+        <v>0.9394946108012314</v>
       </c>
       <c r="T40">
-        <v>0.9904871377410074</v>
+        <v>1.003268729594857</v>
       </c>
     </row>
     <row r="41">
@@ -4331,43 +4331,43 @@
         </is>
       </c>
       <c r="H41">
-        <v>-0.5116146559729645</v>
+        <v>-0.5369591626463901</v>
       </c>
       <c r="I41">
-        <v>0.1871635112221394</v>
+        <v>0.2036126439218424</v>
       </c>
       <c r="J41">
-        <v>0.0138494055627222</v>
+        <v>0.01013807726876701</v>
       </c>
       <c r="K41">
-        <v>-0.5231870318312245</v>
+        <v>-0.5428493951436821</v>
       </c>
       <c r="L41">
-        <v>-0.8514261295155847</v>
+        <v>-0.9272919620447222</v>
       </c>
       <c r="M41">
-        <v>-0.793476231018071</v>
+        <v>-0.8619565639887226</v>
       </c>
       <c r="N41">
-        <v>-0.7360172646291882</v>
+        <v>-0.7876843424006484</v>
       </c>
       <c r="O41">
-        <v>-0.6423676349649825</v>
+        <v>-0.6722046376942312</v>
       </c>
       <c r="P41">
-        <v>-0.5231870318312245</v>
+        <v>-0.5428493951436821</v>
       </c>
       <c r="Q41">
-        <v>-0.3950190029311372</v>
+        <v>-0.4083738360338057</v>
       </c>
       <c r="R41">
-        <v>-0.2624236899512734</v>
+        <v>-0.2757117741559034</v>
       </c>
       <c r="S41">
-        <v>-0.1853170997108407</v>
+        <v>-0.1913649839674343</v>
       </c>
       <c r="T41">
-        <v>-0.1024529610643907</v>
+        <v>-0.1120617046669647</v>
       </c>
     </row>
     <row r="42">
@@ -4401,43 +4401,43 @@
         </is>
       </c>
       <c r="H42">
-        <v>-0.2997581758479709</v>
+        <v>-0.2914665335266804</v>
       </c>
       <c r="I42">
-        <v>0.1205935446563193</v>
+        <v>0.1268638371184199</v>
       </c>
       <c r="J42">
-        <v>0.005808229748890053</v>
+        <v>0.004336999041612884</v>
       </c>
       <c r="K42">
-        <v>-0.3003177394172399</v>
+        <v>-0.2881630288386164</v>
       </c>
       <c r="L42">
-        <v>-0.5470176895445191</v>
+        <v>-0.5529306099134519</v>
       </c>
       <c r="M42">
-        <v>-0.4993147198083546</v>
+        <v>-0.508395418766707</v>
       </c>
       <c r="N42">
-        <v>-0.4494023760354909</v>
+        <v>-0.4551259496182919</v>
       </c>
       <c r="O42">
-        <v>-0.3806903742159381</v>
+        <v>-0.3729647263001437</v>
       </c>
       <c r="P42">
-        <v>-0.3003177394172399</v>
+        <v>-0.2881630288386164</v>
       </c>
       <c r="Q42">
-        <v>-0.2172628751729367</v>
+        <v>-0.2057689564853515</v>
       </c>
       <c r="R42">
-        <v>-0.1437441682113862</v>
+        <v>-0.1312028242246061</v>
       </c>
       <c r="S42">
-        <v>-0.1066270697579693</v>
+        <v>-0.08836986486702653</v>
       </c>
       <c r="T42">
-        <v>-0.07035117526766081</v>
+        <v>-0.05075267660401554</v>
       </c>
     </row>
     <row r="43">
@@ -4471,43 +4471,43 @@
         </is>
       </c>
       <c r="H43">
-        <v>0.5417060408592684</v>
+        <v>0.5336913927167031</v>
       </c>
       <c r="I43">
-        <v>0.2487964918880957</v>
+        <v>0.2519487102677469</v>
       </c>
       <c r="J43">
-        <v>0.02637162723743947</v>
+        <v>0.01807548370186413</v>
       </c>
       <c r="K43">
-        <v>0.5604503041457983</v>
+        <v>0.5420514501089884</v>
       </c>
       <c r="L43">
-        <v>-0.01666641103674497</v>
+        <v>0.01280902634430924</v>
       </c>
       <c r="M43">
-        <v>0.09536507547659817</v>
+        <v>0.1120212086109604</v>
       </c>
       <c r="N43">
-        <v>0.2182271469328651</v>
+        <v>0.2147962563771071</v>
       </c>
       <c r="O43">
-        <v>0.3848421882080577</v>
+        <v>0.3671732564636359</v>
       </c>
       <c r="P43">
-        <v>0.5604503041457983</v>
+        <v>0.5420514501089884</v>
       </c>
       <c r="Q43">
-        <v>0.716696337758487</v>
+        <v>0.7070879191567029</v>
       </c>
       <c r="R43">
-        <v>0.8442323233560615</v>
+        <v>0.8586412762319757</v>
       </c>
       <c r="S43">
-        <v>0.9268458555843748</v>
+        <v>0.9394946108012314</v>
       </c>
       <c r="T43">
-        <v>0.9904871377410074</v>
+        <v>1.003268729594857</v>
       </c>
     </row>
     <row r="44">
@@ -4541,43 +4541,43 @@
         </is>
       </c>
       <c r="H44">
-        <v>-0.2997581758479709</v>
+        <v>-0.2914665335266804</v>
       </c>
       <c r="I44">
-        <v>0.1205935446563193</v>
+        <v>0.1268638371184199</v>
       </c>
       <c r="J44">
-        <v>0.005808229748890053</v>
+        <v>0.004336999041612884</v>
       </c>
       <c r="K44">
-        <v>-0.3003177394172399</v>
+        <v>-0.2881630288386164</v>
       </c>
       <c r="L44">
-        <v>-0.5470176895445191</v>
+        <v>-0.5529306099134519</v>
       </c>
       <c r="M44">
-        <v>-0.4993147198083546</v>
+        <v>-0.508395418766707</v>
       </c>
       <c r="N44">
-        <v>-0.4494023760354909</v>
+        <v>-0.4551259496182919</v>
       </c>
       <c r="O44">
-        <v>-0.3806903742159381</v>
+        <v>-0.3729647263001437</v>
       </c>
       <c r="P44">
-        <v>-0.3003177394172399</v>
+        <v>-0.2881630288386164</v>
       </c>
       <c r="Q44">
-        <v>-0.2172628751729367</v>
+        <v>-0.2057689564853515</v>
       </c>
       <c r="R44">
-        <v>-0.1437441682113862</v>
+        <v>-0.1312028242246061</v>
       </c>
       <c r="S44">
-        <v>-0.1066270697579693</v>
+        <v>-0.08836986486702653</v>
       </c>
       <c r="T44">
-        <v>-0.07035117526766081</v>
+        <v>-0.05075267660401554</v>
       </c>
     </row>
     <row r="45">
@@ -4611,43 +4611,43 @@
         </is>
       </c>
       <c r="H45">
-        <v>0.5417060408592684</v>
+        <v>0.5336913927167031</v>
       </c>
       <c r="I45">
-        <v>0.2487964918880957</v>
+        <v>0.2519487102677469</v>
       </c>
       <c r="J45">
-        <v>0.02637162723743947</v>
+        <v>0.01807548370186413</v>
       </c>
       <c r="K45">
-        <v>0.5604503041457983</v>
+        <v>0.5420514501089884</v>
       </c>
       <c r="L45">
-        <v>-0.01666641103674497</v>
+        <v>0.01280902634430924</v>
       </c>
       <c r="M45">
-        <v>0.09536507547659817</v>
+        <v>0.1120212086109604</v>
       </c>
       <c r="N45">
-        <v>0.2182271469328651</v>
+        <v>0.2147962563771071</v>
       </c>
       <c r="O45">
-        <v>0.3848421882080577</v>
+        <v>0.3671732564636359</v>
       </c>
       <c r="P45">
-        <v>0.5604503041457983</v>
+        <v>0.5420514501089884</v>
       </c>
       <c r="Q45">
-        <v>0.716696337758487</v>
+        <v>0.7070879191567029</v>
       </c>
       <c r="R45">
-        <v>0.8442323233560615</v>
+        <v>0.8586412762319757</v>
       </c>
       <c r="S45">
-        <v>0.9268458555843748</v>
+        <v>0.9394946108012314</v>
       </c>
       <c r="T45">
-        <v>0.9904871377410074</v>
+        <v>1.003268729594857</v>
       </c>
     </row>
     <row r="46">
@@ -4681,43 +4681,43 @@
         </is>
       </c>
       <c r="H46">
-        <v>0.3113032558764295</v>
+        <v>0.3232031014683357</v>
       </c>
       <c r="I46">
-        <v>0.1362093634617424</v>
+        <v>0.1420946102486272</v>
       </c>
       <c r="J46">
-        <v>0.007443507277702275</v>
+        <v>0.005740520804359723</v>
       </c>
       <c r="K46">
-        <v>0.316257303341141</v>
+        <v>0.329737376709393</v>
       </c>
       <c r="L46">
-        <v>0.02694270680745655</v>
+        <v>0.02380958686559168</v>
       </c>
       <c r="M46">
-        <v>0.07529715532475259</v>
+        <v>0.07728212611721173</v>
       </c>
       <c r="N46">
-        <v>0.1330345569714191</v>
+        <v>0.1379085124364979</v>
       </c>
       <c r="O46">
-        <v>0.2230796353816032</v>
+        <v>0.2323905509752022</v>
       </c>
       <c r="P46">
-        <v>0.316257303341141</v>
+        <v>0.329737376709393</v>
       </c>
       <c r="Q46">
-        <v>0.4062321658569829</v>
+        <v>0.4212820878663344</v>
       </c>
       <c r="R46">
-        <v>0.4797921499961845</v>
+        <v>0.4998753731485056</v>
       </c>
       <c r="S46">
-        <v>0.5273055052693616</v>
+        <v>0.5460390596689056</v>
       </c>
       <c r="T46">
-        <v>0.5693657637896794</v>
+        <v>0.5866353602915522</v>
       </c>
     </row>
     <row r="47">
@@ -4751,43 +4751,43 @@
         </is>
       </c>
       <c r="H47">
-        <v>-0.5116146559729645</v>
+        <v>-0.5369591626463901</v>
       </c>
       <c r="I47">
-        <v>0.1871635112221394</v>
+        <v>0.2036126439218424</v>
       </c>
       <c r="J47">
-        <v>0.0138494055627222</v>
+        <v>0.01013807726876701</v>
       </c>
       <c r="K47">
-        <v>-0.5231870318312245</v>
+        <v>-0.5428493951436821</v>
       </c>
       <c r="L47">
-        <v>-0.8514261295155847</v>
+        <v>-0.9272919620447222</v>
       </c>
       <c r="M47">
-        <v>-0.793476231018071</v>
+        <v>-0.8619565639887226</v>
       </c>
       <c r="N47">
-        <v>-0.7360172646291882</v>
+        <v>-0.7876843424006484</v>
       </c>
       <c r="O47">
-        <v>-0.6423676349649825</v>
+        <v>-0.6722046376942312</v>
       </c>
       <c r="P47">
-        <v>-0.5231870318312245</v>
+        <v>-0.5428493951436821</v>
       </c>
       <c r="Q47">
-        <v>-0.3950190029311372</v>
+        <v>-0.4083738360338057</v>
       </c>
       <c r="R47">
-        <v>-0.2624236899512734</v>
+        <v>-0.2757117741559034</v>
       </c>
       <c r="S47">
-        <v>-0.1853170997108407</v>
+        <v>-0.1913649839674343</v>
       </c>
       <c r="T47">
-        <v>-0.1024529610643907</v>
+        <v>-0.1120617046669647</v>
       </c>
     </row>
     <row r="48">
@@ -4821,43 +4821,43 @@
         </is>
       </c>
       <c r="H48">
-        <v>-0.2997581758479709</v>
+        <v>-0.2914665335266804</v>
       </c>
       <c r="I48">
-        <v>0.1205935446563193</v>
+        <v>0.1268638371184199</v>
       </c>
       <c r="J48">
-        <v>0.005808229748890053</v>
+        <v>0.004336999041612884</v>
       </c>
       <c r="K48">
-        <v>-0.3003177394172399</v>
+        <v>-0.2881630288386164</v>
       </c>
       <c r="L48">
-        <v>-0.5470176895445191</v>
+        <v>-0.5529306099134519</v>
       </c>
       <c r="M48">
-        <v>-0.4993147198083546</v>
+        <v>-0.508395418766707</v>
       </c>
       <c r="N48">
-        <v>-0.4494023760354909</v>
+        <v>-0.4551259496182919</v>
       </c>
       <c r="O48">
-        <v>-0.3806903742159381</v>
+        <v>-0.3729647263001437</v>
       </c>
       <c r="P48">
-        <v>-0.3003177394172399</v>
+        <v>-0.2881630288386164</v>
       </c>
       <c r="Q48">
-        <v>-0.2172628751729367</v>
+        <v>-0.2057689564853515</v>
       </c>
       <c r="R48">
-        <v>-0.1437441682113862</v>
+        <v>-0.1312028242246061</v>
       </c>
       <c r="S48">
-        <v>-0.1066270697579693</v>
+        <v>-0.08836986486702653</v>
       </c>
       <c r="T48">
-        <v>-0.07035117526766081</v>
+        <v>-0.05075267660401554</v>
       </c>
     </row>
     <row r="49">
@@ -4891,43 +4891,43 @@
         </is>
       </c>
       <c r="H49">
-        <v>0.5417060408592684</v>
+        <v>0.5336913927167031</v>
       </c>
       <c r="I49">
-        <v>0.2487964918880957</v>
+        <v>0.2519487102677469</v>
       </c>
       <c r="J49">
-        <v>0.02637162723743947</v>
+        <v>0.01807548370186413</v>
       </c>
       <c r="K49">
-        <v>0.5604503041457983</v>
+        <v>0.5420514501089884</v>
       </c>
       <c r="L49">
-        <v>-0.01666641103674497</v>
+        <v>0.01280902634430924</v>
       </c>
       <c r="M49">
-        <v>0.09536507547659817</v>
+        <v>0.1120212086109604</v>
       </c>
       <c r="N49">
-        <v>0.2182271469328651</v>
+        <v>0.2147962563771071</v>
       </c>
       <c r="O49">
-        <v>0.3848421882080577</v>
+        <v>0.3671732564636359</v>
       </c>
       <c r="P49">
-        <v>0.5604503041457983</v>
+        <v>0.5420514501089884</v>
       </c>
       <c r="Q49">
-        <v>0.716696337758487</v>
+        <v>0.7070879191567029</v>
       </c>
       <c r="R49">
-        <v>0.8442323233560615</v>
+        <v>0.8586412762319757</v>
       </c>
       <c r="S49">
-        <v>0.9268458555843748</v>
+        <v>0.9394946108012314</v>
       </c>
       <c r="T49">
-        <v>0.9904871377410074</v>
+        <v>1.003268729594857</v>
       </c>
     </row>
     <row r="50">
@@ -4961,43 +4961,43 @@
         </is>
       </c>
       <c r="H50">
-        <v>0.3113032558764295</v>
+        <v>0.3232031014683357</v>
       </c>
       <c r="I50">
-        <v>0.1362093634617424</v>
+        <v>0.1420946102486272</v>
       </c>
       <c r="J50">
-        <v>0.007443507277702275</v>
+        <v>0.005740520804359723</v>
       </c>
       <c r="K50">
-        <v>0.316257303341141</v>
+        <v>0.329737376709393</v>
       </c>
       <c r="L50">
-        <v>0.02694270680745655</v>
+        <v>0.02380958686559168</v>
       </c>
       <c r="M50">
-        <v>0.07529715532475259</v>
+        <v>0.07728212611721173</v>
       </c>
       <c r="N50">
-        <v>0.1330345569714191</v>
+        <v>0.1379085124364979</v>
       </c>
       <c r="O50">
-        <v>0.2230796353816032</v>
+        <v>0.2323905509752022</v>
       </c>
       <c r="P50">
-        <v>0.316257303341141</v>
+        <v>0.329737376709393</v>
       </c>
       <c r="Q50">
-        <v>0.4062321658569829</v>
+        <v>0.4212820878663344</v>
       </c>
       <c r="R50">
-        <v>0.4797921499961845</v>
+        <v>0.4998753731485056</v>
       </c>
       <c r="S50">
-        <v>0.5273055052693616</v>
+        <v>0.5460390596689056</v>
       </c>
       <c r="T50">
-        <v>0.5693657637896794</v>
+        <v>0.5866353602915522</v>
       </c>
     </row>
     <row r="51">
@@ -5031,43 +5031,43 @@
         </is>
       </c>
       <c r="H51">
-        <v>-0.5116146559729645</v>
+        <v>-0.5369591626463901</v>
       </c>
       <c r="I51">
-        <v>0.1871635112221394</v>
+        <v>0.2036126439218424</v>
       </c>
       <c r="J51">
-        <v>0.0138494055627222</v>
+        <v>0.01013807726876701</v>
       </c>
       <c r="K51">
-        <v>-0.5231870318312245</v>
+        <v>-0.5428493951436821</v>
       </c>
       <c r="L51">
-        <v>-0.8514261295155847</v>
+        <v>-0.9272919620447222</v>
       </c>
       <c r="M51">
-        <v>-0.793476231018071</v>
+        <v>-0.8619565639887226</v>
       </c>
       <c r="N51">
-        <v>-0.7360172646291882</v>
+        <v>-0.7876843424006484</v>
       </c>
       <c r="O51">
-        <v>-0.6423676349649825</v>
+        <v>-0.6722046376942312</v>
       </c>
       <c r="P51">
-        <v>-0.5231870318312245</v>
+        <v>-0.5428493951436821</v>
       </c>
       <c r="Q51">
-        <v>-0.3950190029311372</v>
+        <v>-0.4083738360338057</v>
       </c>
       <c r="R51">
-        <v>-0.2624236899512734</v>
+        <v>-0.2757117741559034</v>
       </c>
       <c r="S51">
-        <v>-0.1853170997108407</v>
+        <v>-0.1913649839674343</v>
       </c>
       <c r="T51">
-        <v>-0.1024529610643907</v>
+        <v>-0.1120617046669647</v>
       </c>
     </row>
     <row r="52">
@@ -5101,43 +5101,43 @@
         </is>
       </c>
       <c r="H52">
-        <v>-0.2997581758479709</v>
+        <v>-0.2914665335266804</v>
       </c>
       <c r="I52">
-        <v>0.1205935446563193</v>
+        <v>0.1268638371184199</v>
       </c>
       <c r="J52">
-        <v>0.005808229748890053</v>
+        <v>0.004336999041612884</v>
       </c>
       <c r="K52">
-        <v>-0.3003177394172399</v>
+        <v>-0.2881630288386164</v>
       </c>
       <c r="L52">
-        <v>-0.5470176895445191</v>
+        <v>-0.5529306099134519</v>
       </c>
       <c r="M52">
-        <v>-0.4993147198083546</v>
+        <v>-0.508395418766707</v>
       </c>
       <c r="N52">
-        <v>-0.4494023760354909</v>
+        <v>-0.4551259496182919</v>
       </c>
       <c r="O52">
-        <v>-0.3806903742159381</v>
+        <v>-0.3729647263001437</v>
       </c>
       <c r="P52">
-        <v>-0.3003177394172399</v>
+        <v>-0.2881630288386164</v>
       </c>
       <c r="Q52">
-        <v>-0.2172628751729367</v>
+        <v>-0.2057689564853515</v>
       </c>
       <c r="R52">
-        <v>-0.1437441682113862</v>
+        <v>-0.1312028242246061</v>
       </c>
       <c r="S52">
-        <v>-0.1066270697579693</v>
+        <v>-0.08836986486702653</v>
       </c>
       <c r="T52">
-        <v>-0.07035117526766081</v>
+        <v>-0.05075267660401554</v>
       </c>
     </row>
     <row r="53">
@@ -5171,43 +5171,43 @@
         </is>
       </c>
       <c r="H53">
-        <v>-1.666137154963477</v>
+        <v>-1.676201540987581</v>
       </c>
       <c r="I53">
-        <v>1.030182074355619</v>
+        <v>1.035283833008518</v>
       </c>
       <c r="J53">
-        <v>0.1084019016706564</v>
+        <v>0.07701312410586839</v>
       </c>
       <c r="K53">
-        <v>-1.628339858179879</v>
+        <v>-1.675147167474839</v>
       </c>
       <c r="L53">
-        <v>-3.870161755723977</v>
+        <v>-3.805123165114205</v>
       </c>
       <c r="M53">
-        <v>-3.488032961964862</v>
+        <v>-3.387966630833503</v>
       </c>
       <c r="N53">
-        <v>-3.003823218096905</v>
+        <v>-2.975243907002977</v>
       </c>
       <c r="O53">
-        <v>-2.290316942476073</v>
+        <v>-2.349070501240922</v>
       </c>
       <c r="P53">
-        <v>-1.628339858179879</v>
+        <v>-1.675147167474839</v>
       </c>
       <c r="Q53">
-        <v>-0.9999871789526356</v>
+        <v>-0.9754761953429016</v>
       </c>
       <c r="R53">
-        <v>-0.2572257762999619</v>
+        <v>-0.183671580782594</v>
       </c>
       <c r="S53">
-        <v>0.03687330688384052</v>
+        <v>0.04702015061722756</v>
       </c>
       <c r="T53">
-        <v>0.1267385224481098</v>
+        <v>0.1771553118029174</v>
       </c>
     </row>
     <row r="54">
@@ -5241,43 +5241,43 @@
         </is>
       </c>
       <c r="H54">
-        <v>0.5417060408592684</v>
+        <v>0.5336913927167031</v>
       </c>
       <c r="I54">
-        <v>0.2487964918880957</v>
+        <v>0.2519487102677469</v>
       </c>
       <c r="J54">
-        <v>0.02637162723743947</v>
+        <v>0.01807548370186413</v>
       </c>
       <c r="K54">
-        <v>0.5604503041457983</v>
+        <v>0.5420514501089884</v>
       </c>
       <c r="L54">
-        <v>-0.01666641103674497</v>
+        <v>0.01280902634430924</v>
       </c>
       <c r="M54">
-        <v>0.09536507547659817</v>
+        <v>0.1120212086109604</v>
       </c>
       <c r="N54">
-        <v>0.2182271469328651</v>
+        <v>0.2147962563771071</v>
       </c>
       <c r="O54">
-        <v>0.3848421882080577</v>
+        <v>0.3671732564636359</v>
       </c>
       <c r="P54">
-        <v>0.5604503041457983</v>
+        <v>0.5420514501089884</v>
       </c>
       <c r="Q54">
-        <v>0.716696337758487</v>
+        <v>0.7070879191567029</v>
       </c>
       <c r="R54">
-        <v>0.8442323233560615</v>
+        <v>0.8586412762319757</v>
       </c>
       <c r="S54">
-        <v>0.9268458555843748</v>
+        <v>0.9394946108012314</v>
       </c>
       <c r="T54">
-        <v>0.9904871377410074</v>
+        <v>1.003268729594857</v>
       </c>
     </row>
     <row r="55">
@@ -5311,43 +5311,43 @@
         </is>
       </c>
       <c r="H55">
-        <v>-0.2997581758479709</v>
+        <v>-0.2914665335266804</v>
       </c>
       <c r="I55">
-        <v>0.1205935446563193</v>
+        <v>0.1268638371184199</v>
       </c>
       <c r="J55">
-        <v>0.005808229748890053</v>
+        <v>0.004336999041612884</v>
       </c>
       <c r="K55">
-        <v>-0.3003177394172399</v>
+        <v>-0.2881630288386164</v>
       </c>
       <c r="L55">
-        <v>-0.5470176895445191</v>
+        <v>-0.5529306099134519</v>
       </c>
       <c r="M55">
-        <v>-0.4993147198083546</v>
+        <v>-0.508395418766707</v>
       </c>
       <c r="N55">
-        <v>-0.4494023760354909</v>
+        <v>-0.4551259496182919</v>
       </c>
       <c r="O55">
-        <v>-0.3806903742159381</v>
+        <v>-0.3729647263001437</v>
       </c>
       <c r="P55">
-        <v>-0.3003177394172399</v>
+        <v>-0.2881630288386164</v>
       </c>
       <c r="Q55">
-        <v>-0.2172628751729367</v>
+        <v>-0.2057689564853515</v>
       </c>
       <c r="R55">
-        <v>-0.1437441682113862</v>
+        <v>-0.1312028242246061</v>
       </c>
       <c r="S55">
-        <v>-0.1066270697579693</v>
+        <v>-0.08836986486702653</v>
       </c>
       <c r="T55">
-        <v>-0.07035117526766081</v>
+        <v>-0.05075267660401554</v>
       </c>
     </row>
     <row r="56">
@@ -5381,43 +5381,43 @@
         </is>
       </c>
       <c r="H56">
-        <v>-0.1046798152858951</v>
+        <v>-0.107017835387122</v>
       </c>
       <c r="I56">
-        <v>0.1301398294968226</v>
+        <v>0.1269459264510429</v>
       </c>
       <c r="J56">
-        <v>0.004489188844228981</v>
+        <v>0.002401968778905081</v>
       </c>
       <c r="K56">
-        <v>-0.1004581502557295</v>
+        <v>-0.1023315305345405</v>
       </c>
       <c r="L56">
-        <v>-0.3753464505385751</v>
+        <v>-0.3681489359962021</v>
       </c>
       <c r="M56">
-        <v>-0.3311505668231341</v>
+        <v>-0.3207942158070026</v>
       </c>
       <c r="N56">
-        <v>-0.2733669922777434</v>
+        <v>-0.2750567385371742</v>
       </c>
       <c r="O56">
-        <v>-0.1881028706283962</v>
+        <v>-0.1909895861441369</v>
       </c>
       <c r="P56">
-        <v>-0.1004581502557295</v>
+        <v>-0.1023315305345405</v>
       </c>
       <c r="Q56">
-        <v>-0.01150899139302317</v>
+        <v>-0.01958741750834391</v>
       </c>
       <c r="R56">
-        <v>0.05620358718629397</v>
+        <v>0.05288336647867456</v>
       </c>
       <c r="S56">
-        <v>0.09790972252884569</v>
+        <v>0.09529479881860209</v>
       </c>
       <c r="T56">
-        <v>0.135475681257319</v>
+        <v>0.1248289554633815</v>
       </c>
     </row>
     <row r="57">
@@ -5451,43 +5451,43 @@
         </is>
       </c>
       <c r="H57">
-        <v>0.5417060408592684</v>
+        <v>0.5336913927167031</v>
       </c>
       <c r="I57">
-        <v>0.2487964918880957</v>
+        <v>0.2519487102677469</v>
       </c>
       <c r="J57">
-        <v>0.02637162723743947</v>
+        <v>0.01807548370186413</v>
       </c>
       <c r="K57">
-        <v>0.5604503041457983</v>
+        <v>0.5420514501089884</v>
       </c>
       <c r="L57">
-        <v>-0.01666641103674497</v>
+        <v>0.01280902634430924</v>
       </c>
       <c r="M57">
-        <v>0.09536507547659817</v>
+        <v>0.1120212086109604</v>
       </c>
       <c r="N57">
-        <v>0.2182271469328651</v>
+        <v>0.2147962563771071</v>
       </c>
       <c r="O57">
-        <v>0.3848421882080577</v>
+        <v>0.3671732564636359</v>
       </c>
       <c r="P57">
-        <v>0.5604503041457983</v>
+        <v>0.5420514501089884</v>
       </c>
       <c r="Q57">
-        <v>0.716696337758487</v>
+        <v>0.7070879191567029</v>
       </c>
       <c r="R57">
-        <v>0.8442323233560615</v>
+        <v>0.8586412762319757</v>
       </c>
       <c r="S57">
-        <v>0.9268458555843748</v>
+        <v>0.9394946108012314</v>
       </c>
       <c r="T57">
-        <v>0.9904871377410074</v>
+        <v>1.003268729594857</v>
       </c>
     </row>
     <row r="58">
@@ -5521,43 +5521,43 @@
         </is>
       </c>
       <c r="H58">
-        <v>-0.1161112990728373</v>
+        <v>-0.1287407946727498</v>
       </c>
       <c r="I58">
-        <v>0.1148021978489128</v>
+        <v>0.1205661088449834</v>
       </c>
       <c r="J58">
-        <v>0.00477873489985893</v>
+        <v>0.004006584006451343</v>
       </c>
       <c r="K58">
-        <v>-0.1133521931553859</v>
+        <v>-0.1273749279336696</v>
       </c>
       <c r="L58">
-        <v>-0.3386719515336633</v>
+        <v>-0.3651564914560492</v>
       </c>
       <c r="M58">
-        <v>-0.3046267419691921</v>
+        <v>-0.3268116841121991</v>
       </c>
       <c r="N58">
-        <v>-0.2621410833031751</v>
+        <v>-0.283057820858777</v>
       </c>
       <c r="O58">
-        <v>-0.1948690341940331</v>
+        <v>-0.2106015902179914</v>
       </c>
       <c r="P58">
-        <v>-0.1133521931553859</v>
+        <v>-0.1273749279336696</v>
       </c>
       <c r="Q58">
-        <v>-0.04023992026320443</v>
+        <v>-0.04965583352737096</v>
       </c>
       <c r="R58">
-        <v>0.02516573387752361</v>
+        <v>0.025814225589536</v>
       </c>
       <c r="S58">
-        <v>0.0687494092616685</v>
+        <v>0.06749840563798652</v>
       </c>
       <c r="T58">
-        <v>0.1091078866312331</v>
+        <v>0.1069579387757273</v>
       </c>
     </row>
     <row r="59">
@@ -5591,43 +5591,43 @@
         </is>
       </c>
       <c r="H59">
-        <v>-0.2997581758479709</v>
+        <v>-0.2914665335266804</v>
       </c>
       <c r="I59">
-        <v>0.1205935446563193</v>
+        <v>0.1268638371184199</v>
       </c>
       <c r="J59">
-        <v>0.005808229748890053</v>
+        <v>0.004336999041612884</v>
       </c>
       <c r="K59">
-        <v>-0.3003177394172399</v>
+        <v>-0.2881630288386164</v>
       </c>
       <c r="L59">
-        <v>-0.5470176895445191</v>
+        <v>-0.5529306099134519</v>
       </c>
       <c r="M59">
-        <v>-0.4993147198083546</v>
+        <v>-0.508395418766707</v>
       </c>
       <c r="N59">
-        <v>-0.4494023760354909</v>
+        <v>-0.4551259496182919</v>
       </c>
       <c r="O59">
-        <v>-0.3806903742159381</v>
+        <v>-0.3729647263001437</v>
       </c>
       <c r="P59">
-        <v>-0.3003177394172399</v>
+        <v>-0.2881630288386164</v>
       </c>
       <c r="Q59">
-        <v>-0.2172628751729367</v>
+        <v>-0.2057689564853515</v>
       </c>
       <c r="R59">
-        <v>-0.1437441682113862</v>
+        <v>-0.1312028242246061</v>
       </c>
       <c r="S59">
-        <v>-0.1066270697579693</v>
+        <v>-0.08836986486702653</v>
       </c>
       <c r="T59">
-        <v>-0.07035117526766081</v>
+        <v>-0.05075267660401554</v>
       </c>
     </row>
     <row r="60">
@@ -5661,43 +5661,43 @@
         </is>
       </c>
       <c r="H60">
-        <v>0.9183909914910773</v>
+        <v>0.9350824013936898</v>
       </c>
       <c r="I60">
-        <v>0.1304830711675759</v>
+        <v>0.1287839575270144</v>
       </c>
       <c r="J60">
-        <v>0.007629190739139556</v>
+        <v>0.004911631260971691</v>
       </c>
       <c r="K60">
-        <v>0.9188769232333426</v>
+        <v>0.9339599256730006</v>
       </c>
       <c r="L60">
-        <v>0.6586142205919907</v>
+        <v>0.6837604478264198</v>
       </c>
       <c r="M60">
-        <v>0.6973144818432745</v>
+        <v>0.7256969263309898</v>
       </c>
       <c r="N60">
-        <v>0.7525626104506297</v>
+        <v>0.7721319863560734</v>
       </c>
       <c r="O60">
-        <v>0.835069406160258</v>
+        <v>0.8480878806056904</v>
       </c>
       <c r="P60">
-        <v>0.9188769232333426</v>
+        <v>0.9339599256730006</v>
       </c>
       <c r="Q60">
-        <v>1.006385161414666</v>
+        <v>1.022096874431145</v>
       </c>
       <c r="R60">
-        <v>1.083930819456203</v>
+        <v>1.09963839975358</v>
       </c>
       <c r="S60">
-        <v>1.134951693682448</v>
+        <v>1.149915295602883</v>
       </c>
       <c r="T60">
-        <v>1.172675806558851</v>
+        <v>1.188425484603933</v>
       </c>
     </row>
     <row r="61">
@@ -5731,43 +5731,43 @@
         </is>
       </c>
       <c r="H61">
-        <v>-0.4065596936517923</v>
+        <v>-0.3861219822456349</v>
       </c>
       <c r="I61">
-        <v>0.1367732975379721</v>
+        <v>0.1375031246846421</v>
       </c>
       <c r="J61">
-        <v>0.007752243424404085</v>
+        <v>0.005396993969338132</v>
       </c>
       <c r="K61">
-        <v>-0.4059009629105702</v>
+        <v>-0.3844796819927853</v>
       </c>
       <c r="L61">
-        <v>-0.6808653523379501</v>
+        <v>-0.660343584330276</v>
       </c>
       <c r="M61">
-        <v>-0.6290055510176999</v>
+        <v>-0.6127355638936063</v>
       </c>
       <c r="N61">
-        <v>-0.5826112935258686</v>
+        <v>-0.5631256427215817</v>
       </c>
       <c r="O61">
-        <v>-0.4980215224411933</v>
+        <v>-0.4774900201554068</v>
       </c>
       <c r="P61">
-        <v>-0.4059009629105702</v>
+        <v>-0.3844796819927853</v>
       </c>
       <c r="Q61">
-        <v>-0.3120138456327275</v>
+        <v>-0.2959074369696905</v>
       </c>
       <c r="R61">
-        <v>-0.2362582856643825</v>
+        <v>-0.2133831762162299</v>
       </c>
       <c r="S61">
-        <v>-0.1875672023811518</v>
+        <v>-0.1617123972455172</v>
       </c>
       <c r="T61">
-        <v>-0.13768853671991</v>
+        <v>-0.1103279673395892</v>
       </c>
     </row>
     <row r="62">
@@ -5801,43 +5801,43 @@
         </is>
       </c>
       <c r="H62">
-        <v>-0.1889578831058645</v>
+        <v>-0.1831147261014914</v>
       </c>
       <c r="I62">
-        <v>0.1327116504290296</v>
+        <v>0.1350369720875784</v>
       </c>
       <c r="J62">
-        <v>0.004988553944890132</v>
+        <v>0.003915876801680832</v>
       </c>
       <c r="K62">
-        <v>-0.1854118738502842</v>
+        <v>-0.1785893086645667</v>
       </c>
       <c r="L62">
-        <v>-0.4602265954673859</v>
+        <v>-0.4649684790586853</v>
       </c>
       <c r="M62">
-        <v>-0.4109149079112364</v>
+        <v>-0.4154883456029336</v>
       </c>
       <c r="N62">
-        <v>-0.3562558322924651</v>
+        <v>-0.358318296277535</v>
       </c>
       <c r="O62">
-        <v>-0.2767524515129072</v>
+        <v>-0.2698399395404846</v>
       </c>
       <c r="P62">
-        <v>-0.1854118738502842</v>
+        <v>-0.1785893086645667</v>
       </c>
       <c r="Q62">
-        <v>-0.09630601969289393</v>
+        <v>-0.09008199488237223</v>
       </c>
       <c r="R62">
-        <v>-0.02334182334123727</v>
+        <v>-0.01445770825028103</v>
       </c>
       <c r="S62">
-        <v>0.02185289638685428</v>
+        <v>0.03175994551138536</v>
       </c>
       <c r="T62">
-        <v>0.0567593032052706</v>
+        <v>0.06508679198580132</v>
       </c>
     </row>
     <row r="63">
@@ -5871,43 +5871,43 @@
         </is>
       </c>
       <c r="H63">
-        <v>0.4928832352681846</v>
+        <v>0.5216747421585012</v>
       </c>
       <c r="I63">
-        <v>0.2081492105235483</v>
+        <v>0.1656690180157772</v>
       </c>
       <c r="J63">
-        <v>0.142336995204372</v>
+        <v>0.06199340762075325</v>
       </c>
       <c r="K63">
-        <v>0.4948766498617353</v>
+        <v>0.4970093760277954</v>
       </c>
       <c r="L63">
-        <v>0.194505971157467</v>
+        <v>0.2544938193727065</v>
       </c>
       <c r="M63">
-        <v>0.214159402191094</v>
+        <v>0.2818463068147971</v>
       </c>
       <c r="N63">
-        <v>0.2338548175674627</v>
+        <v>0.3183431310005265</v>
       </c>
       <c r="O63">
-        <v>0.3454576614088294</v>
+        <v>0.4034339590777929</v>
       </c>
       <c r="P63">
-        <v>0.4948766498617353</v>
+        <v>0.4970093760277954</v>
       </c>
       <c r="Q63">
-        <v>0.5778643295666729</v>
+        <v>0.621124205496744</v>
       </c>
       <c r="R63">
-        <v>0.7787218439451356</v>
+        <v>0.7744348303172901</v>
       </c>
       <c r="S63">
-        <v>0.9380251412749596</v>
+        <v>0.8405695748132813</v>
       </c>
       <c r="T63">
-        <v>1.018700735436573</v>
+        <v>0.867919380982383</v>
       </c>
     </row>
     <row r="64">
@@ -7963,43 +7963,43 @@
         <v>1.06</v>
       </c>
       <c r="F5">
-        <v>1.589311306603231</v>
+        <v>1.589395984848507</v>
       </c>
       <c r="G5">
-        <v>0.007205628292603781</v>
+        <v>0.007262318948204624</v>
       </c>
       <c r="H5">
-        <v>0.0002271076041062111</v>
+        <v>0.0001464555606329597</v>
       </c>
       <c r="I5">
-        <v>1.587119633634973</v>
+        <v>1.587220493981195</v>
       </c>
       <c r="J5">
-        <v>1.582167677340778</v>
+        <v>1.582191212529661</v>
       </c>
       <c r="K5">
-        <v>1.58232864116933</v>
+        <v>1.582405565624905</v>
       </c>
       <c r="L5">
-        <v>1.582751154194213</v>
+        <v>1.582791209486076</v>
       </c>
       <c r="M5">
-        <v>1.584179616121803</v>
+        <v>1.584142124250705</v>
       </c>
       <c r="N5">
-        <v>1.587119633634973</v>
+        <v>1.587220493981195</v>
       </c>
       <c r="O5">
-        <v>1.592126237203439</v>
+        <v>1.592257135192646</v>
       </c>
       <c r="P5">
-        <v>1.598731928006224</v>
+        <v>1.599159409399299</v>
       </c>
       <c r="Q5">
-        <v>1.603723493396287</v>
+        <v>1.604247882397833</v>
       </c>
       <c r="R5">
-        <v>1.608904274809916</v>
+        <v>1.608928520286697</v>
       </c>
     </row>
     <row r="6">
@@ -12461,43 +12461,43 @@
         </is>
       </c>
       <c r="H2">
-        <v>0.5417060408592684</v>
+        <v>0.5336913927167031</v>
       </c>
       <c r="I2">
-        <v>0.2487964918880957</v>
+        <v>0.2519487102677469</v>
       </c>
       <c r="J2">
-        <v>0.02637162723743947</v>
+        <v>0.01807548370186413</v>
       </c>
       <c r="K2">
-        <v>0.5604503041457983</v>
+        <v>0.5420514501089884</v>
       </c>
       <c r="L2">
-        <v>-0.01666641103674497</v>
+        <v>0.01280902634430924</v>
       </c>
       <c r="M2">
-        <v>0.09536507547659817</v>
+        <v>0.1120212086109604</v>
       </c>
       <c r="N2">
-        <v>0.2182271469328651</v>
+        <v>0.2147962563771071</v>
       </c>
       <c r="O2">
-        <v>0.3848421882080577</v>
+        <v>0.3671732564636359</v>
       </c>
       <c r="P2">
-        <v>0.5604503041457983</v>
+        <v>0.5420514501089884</v>
       </c>
       <c r="Q2">
-        <v>0.716696337758487</v>
+        <v>0.7070879191567029</v>
       </c>
       <c r="R2">
-        <v>0.8442323233560615</v>
+        <v>0.8586412762319757</v>
       </c>
       <c r="S2">
-        <v>0.9268458555843748</v>
+        <v>0.9394946108012314</v>
       </c>
       <c r="T2">
-        <v>0.9904871377410074</v>
+        <v>1.003268729594857</v>
       </c>
     </row>
     <row r="3">
@@ -12531,43 +12531,43 @@
         </is>
       </c>
       <c r="H3">
-        <v>-0.5116146559729645</v>
+        <v>-0.5369591626463901</v>
       </c>
       <c r="I3">
-        <v>0.1871635112221394</v>
+        <v>0.2036126439218424</v>
       </c>
       <c r="J3">
-        <v>0.0138494055627222</v>
+        <v>0.01013807726876701</v>
       </c>
       <c r="K3">
-        <v>-0.5231870318312245</v>
+        <v>-0.5428493951436821</v>
       </c>
       <c r="L3">
-        <v>-0.8514261295155847</v>
+        <v>-0.9272919620447222</v>
       </c>
       <c r="M3">
-        <v>-0.793476231018071</v>
+        <v>-0.8619565639887226</v>
       </c>
       <c r="N3">
-        <v>-0.7360172646291882</v>
+        <v>-0.7876843424006484</v>
       </c>
       <c r="O3">
-        <v>-0.6423676349649825</v>
+        <v>-0.6722046376942312</v>
       </c>
       <c r="P3">
-        <v>-0.5231870318312245</v>
+        <v>-0.5428493951436821</v>
       </c>
       <c r="Q3">
-        <v>-0.3950190029311372</v>
+        <v>-0.4083738360338057</v>
       </c>
       <c r="R3">
-        <v>-0.2624236899512734</v>
+        <v>-0.2757117741559034</v>
       </c>
       <c r="S3">
-        <v>-0.1853170997108407</v>
+        <v>-0.1913649839674343</v>
       </c>
       <c r="T3">
-        <v>-0.1024529610643907</v>
+        <v>-0.1120617046669647</v>
       </c>
     </row>
     <row r="4">
@@ -12601,43 +12601,43 @@
         </is>
       </c>
       <c r="H4">
-        <v>-0.2997581758479709</v>
+        <v>-0.2914665335266804</v>
       </c>
       <c r="I4">
-        <v>0.1205935446563193</v>
+        <v>0.1268638371184199</v>
       </c>
       <c r="J4">
-        <v>0.005808229748890053</v>
+        <v>0.004336999041612884</v>
       </c>
       <c r="K4">
-        <v>-0.3003177394172399</v>
+        <v>-0.2881630288386164</v>
       </c>
       <c r="L4">
-        <v>-0.5470176895445191</v>
+        <v>-0.5529306099134519</v>
       </c>
       <c r="M4">
-        <v>-0.4993147198083546</v>
+        <v>-0.508395418766707</v>
       </c>
       <c r="N4">
-        <v>-0.4494023760354909</v>
+        <v>-0.4551259496182919</v>
       </c>
       <c r="O4">
-        <v>-0.3806903742159381</v>
+        <v>-0.3729647263001437</v>
       </c>
       <c r="P4">
-        <v>-0.3003177394172399</v>
+        <v>-0.2881630288386164</v>
       </c>
       <c r="Q4">
-        <v>-0.2172628751729367</v>
+        <v>-0.2057689564853515</v>
       </c>
       <c r="R4">
-        <v>-0.1437441682113862</v>
+        <v>-0.1312028242246061</v>
       </c>
       <c r="S4">
-        <v>-0.1066270697579693</v>
+        <v>-0.08836986486702653</v>
       </c>
       <c r="T4">
-        <v>-0.07035117526766081</v>
+        <v>-0.05075267660401554</v>
       </c>
     </row>
     <row r="5">
@@ -12671,43 +12671,43 @@
         </is>
       </c>
       <c r="H5">
-        <v>0.5417060408592684</v>
+        <v>0.5336913927167031</v>
       </c>
       <c r="I5">
-        <v>0.2487964918880957</v>
+        <v>0.2519487102677469</v>
       </c>
       <c r="J5">
-        <v>0.02637162723743947</v>
+        <v>0.01807548370186413</v>
       </c>
       <c r="K5">
-        <v>0.5604503041457983</v>
+        <v>0.5420514501089884</v>
       </c>
       <c r="L5">
-        <v>-0.01666641103674497</v>
+        <v>0.01280902634430924</v>
       </c>
       <c r="M5">
-        <v>0.09536507547659817</v>
+        <v>0.1120212086109604</v>
       </c>
       <c r="N5">
-        <v>0.2182271469328651</v>
+        <v>0.2147962563771071</v>
       </c>
       <c r="O5">
-        <v>0.3848421882080577</v>
+        <v>0.3671732564636359</v>
       </c>
       <c r="P5">
-        <v>0.5604503041457983</v>
+        <v>0.5420514501089884</v>
       </c>
       <c r="Q5">
-        <v>0.716696337758487</v>
+        <v>0.7070879191567029</v>
       </c>
       <c r="R5">
-        <v>0.8442323233560615</v>
+        <v>0.8586412762319757</v>
       </c>
       <c r="S5">
-        <v>0.9268458555843748</v>
+        <v>0.9394946108012314</v>
       </c>
       <c r="T5">
-        <v>0.9904871377410074</v>
+        <v>1.003268729594857</v>
       </c>
     </row>
     <row r="6">
@@ -12741,43 +12741,43 @@
         </is>
       </c>
       <c r="H6">
-        <v>-0.2997581758479709</v>
+        <v>-0.2914665335266804</v>
       </c>
       <c r="I6">
-        <v>0.1205935446563193</v>
+        <v>0.1268638371184199</v>
       </c>
       <c r="J6">
-        <v>0.005808229748890053</v>
+        <v>0.004336999041612884</v>
       </c>
       <c r="K6">
-        <v>-0.3003177394172399</v>
+        <v>-0.2881630288386164</v>
       </c>
       <c r="L6">
-        <v>-0.5470176895445191</v>
+        <v>-0.5529306099134519</v>
       </c>
       <c r="M6">
-        <v>-0.4993147198083546</v>
+        <v>-0.508395418766707</v>
       </c>
       <c r="N6">
-        <v>-0.4494023760354909</v>
+        <v>-0.4551259496182919</v>
       </c>
       <c r="O6">
-        <v>-0.3806903742159381</v>
+        <v>-0.3729647263001437</v>
       </c>
       <c r="P6">
-        <v>-0.3003177394172399</v>
+        <v>-0.2881630288386164</v>
       </c>
       <c r="Q6">
-        <v>-0.2172628751729367</v>
+        <v>-0.2057689564853515</v>
       </c>
       <c r="R6">
-        <v>-0.1437441682113862</v>
+        <v>-0.1312028242246061</v>
       </c>
       <c r="S6">
-        <v>-0.1066270697579693</v>
+        <v>-0.08836986486702653</v>
       </c>
       <c r="T6">
-        <v>-0.07035117526766081</v>
+        <v>-0.05075267660401554</v>
       </c>
     </row>
     <row r="7">
@@ -12811,43 +12811,43 @@
         </is>
       </c>
       <c r="H7">
-        <v>0.5417060408592684</v>
+        <v>0.5336913927167031</v>
       </c>
       <c r="I7">
-        <v>0.2487964918880957</v>
+        <v>0.2519487102677469</v>
       </c>
       <c r="J7">
-        <v>0.02637162723743947</v>
+        <v>0.01807548370186413</v>
       </c>
       <c r="K7">
-        <v>0.5604503041457983</v>
+        <v>0.5420514501089884</v>
       </c>
       <c r="L7">
-        <v>-0.01666641103674497</v>
+        <v>0.01280902634430924</v>
       </c>
       <c r="M7">
-        <v>0.09536507547659817</v>
+        <v>0.1120212086109604</v>
       </c>
       <c r="N7">
-        <v>0.2182271469328651</v>
+        <v>0.2147962563771071</v>
       </c>
       <c r="O7">
-        <v>0.3848421882080577</v>
+        <v>0.3671732564636359</v>
       </c>
       <c r="P7">
-        <v>0.5604503041457983</v>
+        <v>0.5420514501089884</v>
       </c>
       <c r="Q7">
-        <v>0.716696337758487</v>
+        <v>0.7070879191567029</v>
       </c>
       <c r="R7">
-        <v>0.8442323233560615</v>
+        <v>0.8586412762319757</v>
       </c>
       <c r="S7">
-        <v>0.9268458555843748</v>
+        <v>0.9394946108012314</v>
       </c>
       <c r="T7">
-        <v>0.9904871377410074</v>
+        <v>1.003268729594857</v>
       </c>
     </row>
     <row r="8">
@@ -12881,43 +12881,43 @@
         </is>
       </c>
       <c r="H8">
-        <v>0.3113032558764295</v>
+        <v>0.3232031014683357</v>
       </c>
       <c r="I8">
-        <v>0.1362093634617424</v>
+        <v>0.1420946102486272</v>
       </c>
       <c r="J8">
-        <v>0.007443507277702275</v>
+        <v>0.005740520804359723</v>
       </c>
       <c r="K8">
-        <v>0.316257303341141</v>
+        <v>0.329737376709393</v>
       </c>
       <c r="L8">
-        <v>0.02694270680745655</v>
+        <v>0.02380958686559168</v>
       </c>
       <c r="M8">
-        <v>0.07529715532475259</v>
+        <v>0.07728212611721173</v>
       </c>
       <c r="N8">
-        <v>0.1330345569714191</v>
+        <v>0.1379085124364979</v>
       </c>
       <c r="O8">
-        <v>0.2230796353816032</v>
+        <v>0.2323905509752022</v>
       </c>
       <c r="P8">
-        <v>0.316257303341141</v>
+        <v>0.329737376709393</v>
       </c>
       <c r="Q8">
-        <v>0.4062321658569829</v>
+        <v>0.4212820878663344</v>
       </c>
       <c r="R8">
-        <v>0.4797921499961845</v>
+        <v>0.4998753731485056</v>
       </c>
       <c r="S8">
-        <v>0.5273055052693616</v>
+        <v>0.5460390596689056</v>
       </c>
       <c r="T8">
-        <v>0.5693657637896794</v>
+        <v>0.5866353602915522</v>
       </c>
     </row>
     <row r="9">
@@ -12951,43 +12951,43 @@
         </is>
       </c>
       <c r="H9">
-        <v>-0.5116146559729645</v>
+        <v>-0.5369591626463901</v>
       </c>
       <c r="I9">
-        <v>0.1871635112221394</v>
+        <v>0.2036126439218424</v>
       </c>
       <c r="J9">
-        <v>0.0138494055627222</v>
+        <v>0.01013807726876701</v>
       </c>
       <c r="K9">
-        <v>-0.5231870318312245</v>
+        <v>-0.5428493951436821</v>
       </c>
       <c r="L9">
-        <v>-0.8514261295155847</v>
+        <v>-0.9272919620447222</v>
       </c>
       <c r="M9">
-        <v>-0.793476231018071</v>
+        <v>-0.8619565639887226</v>
       </c>
       <c r="N9">
-        <v>-0.7360172646291882</v>
+        <v>-0.7876843424006484</v>
       </c>
       <c r="O9">
-        <v>-0.6423676349649825</v>
+        <v>-0.6722046376942312</v>
       </c>
       <c r="P9">
-        <v>-0.5231870318312245</v>
+        <v>-0.5428493951436821</v>
       </c>
       <c r="Q9">
-        <v>-0.3950190029311372</v>
+        <v>-0.4083738360338057</v>
       </c>
       <c r="R9">
-        <v>-0.2624236899512734</v>
+        <v>-0.2757117741559034</v>
       </c>
       <c r="S9">
-        <v>-0.1853170997108407</v>
+        <v>-0.1913649839674343</v>
       </c>
       <c r="T9">
-        <v>-0.1024529610643907</v>
+        <v>-0.1120617046669647</v>
       </c>
     </row>
     <row r="10">
@@ -13021,43 +13021,43 @@
         </is>
       </c>
       <c r="H10">
-        <v>-0.2997581758479709</v>
+        <v>-0.2914665335266804</v>
       </c>
       <c r="I10">
-        <v>0.1205935446563193</v>
+        <v>0.1268638371184199</v>
       </c>
       <c r="J10">
-        <v>0.005808229748890053</v>
+        <v>0.004336999041612884</v>
       </c>
       <c r="K10">
-        <v>-0.3003177394172399</v>
+        <v>-0.2881630288386164</v>
       </c>
       <c r="L10">
-        <v>-0.5470176895445191</v>
+        <v>-0.5529306099134519</v>
       </c>
       <c r="M10">
-        <v>-0.4993147198083546</v>
+        <v>-0.508395418766707</v>
       </c>
       <c r="N10">
-        <v>-0.4494023760354909</v>
+        <v>-0.4551259496182919</v>
       </c>
       <c r="O10">
-        <v>-0.3806903742159381</v>
+        <v>-0.3729647263001437</v>
       </c>
       <c r="P10">
-        <v>-0.3003177394172399</v>
+        <v>-0.2881630288386164</v>
       </c>
       <c r="Q10">
-        <v>-0.2172628751729367</v>
+        <v>-0.2057689564853515</v>
       </c>
       <c r="R10">
-        <v>-0.1437441682113862</v>
+        <v>-0.1312028242246061</v>
       </c>
       <c r="S10">
-        <v>-0.1066270697579693</v>
+        <v>-0.08836986486702653</v>
       </c>
       <c r="T10">
-        <v>-0.07035117526766081</v>
+        <v>-0.05075267660401554</v>
       </c>
     </row>
     <row r="11">
@@ -13091,43 +13091,43 @@
         </is>
       </c>
       <c r="H11">
-        <v>0.5417060408592684</v>
+        <v>0.5336913927167031</v>
       </c>
       <c r="I11">
-        <v>0.2487964918880957</v>
+        <v>0.2519487102677469</v>
       </c>
       <c r="J11">
-        <v>0.02637162723743947</v>
+        <v>0.01807548370186413</v>
       </c>
       <c r="K11">
-        <v>0.5604503041457983</v>
+        <v>0.5420514501089884</v>
       </c>
       <c r="L11">
-        <v>-0.01666641103674497</v>
+        <v>0.01280902634430924</v>
       </c>
       <c r="M11">
-        <v>0.09536507547659817</v>
+        <v>0.1120212086109604</v>
       </c>
       <c r="N11">
-        <v>0.2182271469328651</v>
+        <v>0.2147962563771071</v>
       </c>
       <c r="O11">
-        <v>0.3848421882080577</v>
+        <v>0.3671732564636359</v>
       </c>
       <c r="P11">
-        <v>0.5604503041457983</v>
+        <v>0.5420514501089884</v>
       </c>
       <c r="Q11">
-        <v>0.716696337758487</v>
+        <v>0.7070879191567029</v>
       </c>
       <c r="R11">
-        <v>0.8442323233560615</v>
+        <v>0.8586412762319757</v>
       </c>
       <c r="S11">
-        <v>0.9268458555843748</v>
+        <v>0.9394946108012314</v>
       </c>
       <c r="T11">
-        <v>0.9904871377410074</v>
+        <v>1.003268729594857</v>
       </c>
     </row>
     <row r="12">
@@ -13161,43 +13161,43 @@
         </is>
       </c>
       <c r="H12">
-        <v>0.3113032558764295</v>
+        <v>0.3232031014683357</v>
       </c>
       <c r="I12">
-        <v>0.1362093634617424</v>
+        <v>0.1420946102486272</v>
       </c>
       <c r="J12">
-        <v>0.007443507277702275</v>
+        <v>0.005740520804359723</v>
       </c>
       <c r="K12">
-        <v>0.316257303341141</v>
+        <v>0.329737376709393</v>
       </c>
       <c r="L12">
-        <v>0.02694270680745655</v>
+        <v>0.02380958686559168</v>
       </c>
       <c r="M12">
-        <v>0.07529715532475259</v>
+        <v>0.07728212611721173</v>
       </c>
       <c r="N12">
-        <v>0.1330345569714191</v>
+        <v>0.1379085124364979</v>
       </c>
       <c r="O12">
-        <v>0.2230796353816032</v>
+        <v>0.2323905509752022</v>
       </c>
       <c r="P12">
-        <v>0.316257303341141</v>
+        <v>0.329737376709393</v>
       </c>
       <c r="Q12">
-        <v>0.4062321658569829</v>
+        <v>0.4212820878663344</v>
       </c>
       <c r="R12">
-        <v>0.4797921499961845</v>
+        <v>0.4998753731485056</v>
       </c>
       <c r="S12">
-        <v>0.5273055052693616</v>
+        <v>0.5460390596689056</v>
       </c>
       <c r="T12">
-        <v>0.5693657637896794</v>
+        <v>0.5866353602915522</v>
       </c>
     </row>
     <row r="13">
@@ -13231,43 +13231,43 @@
         </is>
       </c>
       <c r="H13">
-        <v>-0.5116146559729645</v>
+        <v>-0.5369591626463901</v>
       </c>
       <c r="I13">
-        <v>0.1871635112221394</v>
+        <v>0.2036126439218424</v>
       </c>
       <c r="J13">
-        <v>0.0138494055627222</v>
+        <v>0.01013807726876701</v>
       </c>
       <c r="K13">
-        <v>-0.5231870318312245</v>
+        <v>-0.5428493951436821</v>
       </c>
       <c r="L13">
-        <v>-0.8514261295155847</v>
+        <v>-0.9272919620447222</v>
       </c>
       <c r="M13">
-        <v>-0.793476231018071</v>
+        <v>-0.8619565639887226</v>
       </c>
       <c r="N13">
-        <v>-0.7360172646291882</v>
+        <v>-0.7876843424006484</v>
       </c>
       <c r="O13">
-        <v>-0.6423676349649825</v>
+        <v>-0.6722046376942312</v>
       </c>
       <c r="P13">
-        <v>-0.5231870318312245</v>
+        <v>-0.5428493951436821</v>
       </c>
       <c r="Q13">
-        <v>-0.3950190029311372</v>
+        <v>-0.4083738360338057</v>
       </c>
       <c r="R13">
-        <v>-0.2624236899512734</v>
+        <v>-0.2757117741559034</v>
       </c>
       <c r="S13">
-        <v>-0.1853170997108407</v>
+        <v>-0.1913649839674343</v>
       </c>
       <c r="T13">
-        <v>-0.1024529610643907</v>
+        <v>-0.1120617046669647</v>
       </c>
     </row>
     <row r="14">
@@ -13301,43 +13301,43 @@
         </is>
       </c>
       <c r="H14">
-        <v>-0.2997581758479709</v>
+        <v>-0.2914665335266804</v>
       </c>
       <c r="I14">
-        <v>0.1205935446563193</v>
+        <v>0.1268638371184199</v>
       </c>
       <c r="J14">
-        <v>0.005808229748890053</v>
+        <v>0.004336999041612884</v>
       </c>
       <c r="K14">
-        <v>-0.3003177394172399</v>
+        <v>-0.2881630288386164</v>
       </c>
       <c r="L14">
-        <v>-0.5470176895445191</v>
+        <v>-0.5529306099134519</v>
       </c>
       <c r="M14">
-        <v>-0.4993147198083546</v>
+        <v>-0.508395418766707</v>
       </c>
       <c r="N14">
-        <v>-0.4494023760354909</v>
+        <v>-0.4551259496182919</v>
       </c>
       <c r="O14">
-        <v>-0.3806903742159381</v>
+        <v>-0.3729647263001437</v>
       </c>
       <c r="P14">
-        <v>-0.3003177394172399</v>
+        <v>-0.2881630288386164</v>
       </c>
       <c r="Q14">
-        <v>-0.2172628751729367</v>
+        <v>-0.2057689564853515</v>
       </c>
       <c r="R14">
-        <v>-0.1437441682113862</v>
+        <v>-0.1312028242246061</v>
       </c>
       <c r="S14">
-        <v>-0.1066270697579693</v>
+        <v>-0.08836986486702653</v>
       </c>
       <c r="T14">
-        <v>-0.07035117526766081</v>
+        <v>-0.05075267660401554</v>
       </c>
     </row>
     <row r="15">
@@ -13371,43 +13371,43 @@
         </is>
       </c>
       <c r="H15">
-        <v>-1.666137154963477</v>
+        <v>-1.676201540987581</v>
       </c>
       <c r="I15">
-        <v>1.030182074355619</v>
+        <v>1.035283833008518</v>
       </c>
       <c r="J15">
-        <v>0.1084019016706564</v>
+        <v>0.07701312410586839</v>
       </c>
       <c r="K15">
-        <v>-1.628339858179879</v>
+        <v>-1.675147167474839</v>
       </c>
       <c r="L15">
-        <v>-3.870161755723977</v>
+        <v>-3.805123165114205</v>
       </c>
       <c r="M15">
-        <v>-3.488032961964862</v>
+        <v>-3.387966630833503</v>
       </c>
       <c r="N15">
-        <v>-3.003823218096905</v>
+        <v>-2.975243907002977</v>
       </c>
       <c r="O15">
-        <v>-2.290316942476073</v>
+        <v>-2.349070501240922</v>
       </c>
       <c r="P15">
-        <v>-1.628339858179879</v>
+        <v>-1.675147167474839</v>
       </c>
       <c r="Q15">
-        <v>-0.9999871789526356</v>
+        <v>-0.9754761953429016</v>
       </c>
       <c r="R15">
-        <v>-0.2572257762999619</v>
+        <v>-0.183671580782594</v>
       </c>
       <c r="S15">
-        <v>0.03687330688384052</v>
+        <v>0.04702015061722756</v>
       </c>
       <c r="T15">
-        <v>0.1267385224481098</v>
+        <v>0.1771553118029174</v>
       </c>
     </row>
     <row r="16">
@@ -13441,43 +13441,43 @@
         </is>
       </c>
       <c r="H16">
-        <v>0.5417060408592684</v>
+        <v>0.5336913927167031</v>
       </c>
       <c r="I16">
-        <v>0.2487964918880957</v>
+        <v>0.2519487102677469</v>
       </c>
       <c r="J16">
-        <v>0.02637162723743947</v>
+        <v>0.01807548370186413</v>
       </c>
       <c r="K16">
-        <v>0.5604503041457983</v>
+        <v>0.5420514501089884</v>
       </c>
       <c r="L16">
-        <v>-0.01666641103674497</v>
+        <v>0.01280902634430924</v>
       </c>
       <c r="M16">
-        <v>0.09536507547659817</v>
+        <v>0.1120212086109604</v>
       </c>
       <c r="N16">
-        <v>0.2182271469328651</v>
+        <v>0.2147962563771071</v>
       </c>
       <c r="O16">
-        <v>0.3848421882080577</v>
+        <v>0.3671732564636359</v>
       </c>
       <c r="P16">
-        <v>0.5604503041457983</v>
+        <v>0.5420514501089884</v>
       </c>
       <c r="Q16">
-        <v>0.716696337758487</v>
+        <v>0.7070879191567029</v>
       </c>
       <c r="R16">
-        <v>0.8442323233560615</v>
+        <v>0.8586412762319757</v>
       </c>
       <c r="S16">
-        <v>0.9268458555843748</v>
+        <v>0.9394946108012314</v>
       </c>
       <c r="T16">
-        <v>0.9904871377410074</v>
+        <v>1.003268729594857</v>
       </c>
     </row>
     <row r="17">
@@ -13511,43 +13511,43 @@
         </is>
       </c>
       <c r="H17">
-        <v>-0.2997581758479709</v>
+        <v>-0.2914665335266804</v>
       </c>
       <c r="I17">
-        <v>0.1205935446563193</v>
+        <v>0.1268638371184199</v>
       </c>
       <c r="J17">
-        <v>0.005808229748890053</v>
+        <v>0.004336999041612884</v>
       </c>
       <c r="K17">
-        <v>-0.3003177394172399</v>
+        <v>-0.2881630288386164</v>
       </c>
       <c r="L17">
-        <v>-0.5470176895445191</v>
+        <v>-0.5529306099134519</v>
       </c>
       <c r="M17">
-        <v>-0.4993147198083546</v>
+        <v>-0.508395418766707</v>
       </c>
       <c r="N17">
-        <v>-0.4494023760354909</v>
+        <v>-0.4551259496182919</v>
       </c>
       <c r="O17">
-        <v>-0.3806903742159381</v>
+        <v>-0.3729647263001437</v>
       </c>
       <c r="P17">
-        <v>-0.3003177394172399</v>
+        <v>-0.2881630288386164</v>
       </c>
       <c r="Q17">
-        <v>-0.2172628751729367</v>
+        <v>-0.2057689564853515</v>
       </c>
       <c r="R17">
-        <v>-0.1437441682113862</v>
+        <v>-0.1312028242246061</v>
       </c>
       <c r="S17">
-        <v>-0.1066270697579693</v>
+        <v>-0.08836986486702653</v>
       </c>
       <c r="T17">
-        <v>-0.07035117526766081</v>
+        <v>-0.05075267660401554</v>
       </c>
     </row>
     <row r="18">
@@ -13581,43 +13581,43 @@
         </is>
       </c>
       <c r="H18">
-        <v>-0.1046798152858951</v>
+        <v>-0.107017835387122</v>
       </c>
       <c r="I18">
-        <v>0.1301398294968226</v>
+        <v>0.1269459264510429</v>
       </c>
       <c r="J18">
-        <v>0.004489188844228981</v>
+        <v>0.002401968778905081</v>
       </c>
       <c r="K18">
-        <v>-0.1004581502557295</v>
+        <v>-0.1023315305345405</v>
       </c>
       <c r="L18">
-        <v>-0.3753464505385751</v>
+        <v>-0.3681489359962021</v>
       </c>
       <c r="M18">
-        <v>-0.3311505668231341</v>
+        <v>-0.3207942158070026</v>
       </c>
       <c r="N18">
-        <v>-0.2733669922777434</v>
+        <v>-0.2750567385371742</v>
       </c>
       <c r="O18">
-        <v>-0.1881028706283962</v>
+        <v>-0.1909895861441369</v>
       </c>
       <c r="P18">
-        <v>-0.1004581502557295</v>
+        <v>-0.1023315305345405</v>
       </c>
       <c r="Q18">
-        <v>-0.01150899139302317</v>
+        <v>-0.01958741750834391</v>
       </c>
       <c r="R18">
-        <v>0.05620358718629397</v>
+        <v>0.05288336647867456</v>
       </c>
       <c r="S18">
-        <v>0.09790972252884569</v>
+        <v>0.09529479881860209</v>
       </c>
       <c r="T18">
-        <v>0.135475681257319</v>
+        <v>0.1248289554633815</v>
       </c>
     </row>
     <row r="19">
@@ -13651,43 +13651,43 @@
         </is>
       </c>
       <c r="H19">
-        <v>0.5417060408592684</v>
+        <v>0.5336913927167031</v>
       </c>
       <c r="I19">
-        <v>0.2487964918880957</v>
+        <v>0.2519487102677469</v>
       </c>
       <c r="J19">
-        <v>0.02637162723743947</v>
+        <v>0.01807548370186413</v>
       </c>
       <c r="K19">
-        <v>0.5604503041457983</v>
+        <v>0.5420514501089884</v>
       </c>
       <c r="L19">
-        <v>-0.01666641103674497</v>
+        <v>0.01280902634430924</v>
       </c>
       <c r="M19">
-        <v>0.09536507547659817</v>
+        <v>0.1120212086109604</v>
       </c>
       <c r="N19">
-        <v>0.2182271469328651</v>
+        <v>0.2147962563771071</v>
       </c>
       <c r="O19">
-        <v>0.3848421882080577</v>
+        <v>0.3671732564636359</v>
       </c>
       <c r="P19">
-        <v>0.5604503041457983</v>
+        <v>0.5420514501089884</v>
       </c>
       <c r="Q19">
-        <v>0.716696337758487</v>
+        <v>0.7070879191567029</v>
       </c>
       <c r="R19">
-        <v>0.8442323233560615</v>
+        <v>0.8586412762319757</v>
       </c>
       <c r="S19">
-        <v>0.9268458555843748</v>
+        <v>0.9394946108012314</v>
       </c>
       <c r="T19">
-        <v>0.9904871377410074</v>
+        <v>1.003268729594857</v>
       </c>
     </row>
     <row r="20">
@@ -13721,43 +13721,43 @@
         </is>
       </c>
       <c r="H20">
-        <v>-0.1161112990728373</v>
+        <v>-0.1287407946727498</v>
       </c>
       <c r="I20">
-        <v>0.1148021978489128</v>
+        <v>0.1205661088449834</v>
       </c>
       <c r="J20">
-        <v>0.00477873489985893</v>
+        <v>0.004006584006451343</v>
       </c>
       <c r="K20">
-        <v>-0.1133521931553859</v>
+        <v>-0.1273749279336696</v>
       </c>
       <c r="L20">
-        <v>-0.3386719515336633</v>
+        <v>-0.3651564914560492</v>
       </c>
       <c r="M20">
-        <v>-0.3046267419691921</v>
+        <v>-0.3268116841121991</v>
       </c>
       <c r="N20">
-        <v>-0.2621410833031751</v>
+        <v>-0.283057820858777</v>
       </c>
       <c r="O20">
-        <v>-0.1948690341940331</v>
+        <v>-0.2106015902179914</v>
       </c>
       <c r="P20">
-        <v>-0.1133521931553859</v>
+        <v>-0.1273749279336696</v>
       </c>
       <c r="Q20">
-        <v>-0.04023992026320443</v>
+        <v>-0.04965583352737096</v>
       </c>
       <c r="R20">
-        <v>0.02516573387752361</v>
+        <v>0.025814225589536</v>
       </c>
       <c r="S20">
-        <v>0.0687494092616685</v>
+        <v>0.06749840563798652</v>
       </c>
       <c r="T20">
-        <v>0.1091078866312331</v>
+        <v>0.1069579387757273</v>
       </c>
     </row>
     <row r="21">
@@ -13791,43 +13791,43 @@
         </is>
       </c>
       <c r="H21">
-        <v>-0.2997581758479709</v>
+        <v>-0.2914665335266804</v>
       </c>
       <c r="I21">
-        <v>0.1205935446563193</v>
+        <v>0.1268638371184199</v>
       </c>
       <c r="J21">
-        <v>0.005808229748890053</v>
+        <v>0.004336999041612884</v>
       </c>
       <c r="K21">
-        <v>-0.3003177394172399</v>
+        <v>-0.2881630288386164</v>
       </c>
       <c r="L21">
-        <v>-0.5470176895445191</v>
+        <v>-0.5529306099134519</v>
       </c>
       <c r="M21">
-        <v>-0.4993147198083546</v>
+        <v>-0.508395418766707</v>
       </c>
       <c r="N21">
-        <v>-0.4494023760354909</v>
+        <v>-0.4551259496182919</v>
       </c>
       <c r="O21">
-        <v>-0.3806903742159381</v>
+        <v>-0.3729647263001437</v>
       </c>
       <c r="P21">
-        <v>-0.3003177394172399</v>
+        <v>-0.2881630288386164</v>
       </c>
       <c r="Q21">
-        <v>-0.2172628751729367</v>
+        <v>-0.2057689564853515</v>
       </c>
       <c r="R21">
-        <v>-0.1437441682113862</v>
+        <v>-0.1312028242246061</v>
       </c>
       <c r="S21">
-        <v>-0.1066270697579693</v>
+        <v>-0.08836986486702653</v>
       </c>
       <c r="T21">
-        <v>-0.07035117526766081</v>
+        <v>-0.05075267660401554</v>
       </c>
     </row>
     <row r="22">
@@ -13861,43 +13861,43 @@
         </is>
       </c>
       <c r="H22">
-        <v>0.9183909914910773</v>
+        <v>0.9350824013936898</v>
       </c>
       <c r="I22">
-        <v>0.1304830711675759</v>
+        <v>0.1287839575270144</v>
       </c>
       <c r="J22">
-        <v>0.007629190739139556</v>
+        <v>0.004911631260971691</v>
       </c>
       <c r="K22">
-        <v>0.9188769232333426</v>
+        <v>0.9339599256730006</v>
       </c>
       <c r="L22">
-        <v>0.6586142205919907</v>
+        <v>0.6837604478264198</v>
       </c>
       <c r="M22">
-        <v>0.6973144818432745</v>
+        <v>0.7256969263309898</v>
       </c>
       <c r="N22">
-        <v>0.7525626104506297</v>
+        <v>0.7721319863560734</v>
       </c>
       <c r="O22">
-        <v>0.835069406160258</v>
+        <v>0.8480878806056904</v>
       </c>
       <c r="P22">
-        <v>0.9188769232333426</v>
+        <v>0.9339599256730006</v>
       </c>
       <c r="Q22">
-        <v>1.006385161414666</v>
+        <v>1.022096874431145</v>
       </c>
       <c r="R22">
-        <v>1.083930819456203</v>
+        <v>1.09963839975358</v>
       </c>
       <c r="S22">
-        <v>1.134951693682448</v>
+        <v>1.149915295602883</v>
       </c>
       <c r="T22">
-        <v>1.172675806558851</v>
+        <v>1.188425484603933</v>
       </c>
     </row>
     <row r="23">
@@ -13931,43 +13931,43 @@
         </is>
       </c>
       <c r="H23">
-        <v>-0.4065596936517923</v>
+        <v>-0.3861219822456349</v>
       </c>
       <c r="I23">
-        <v>0.1367732975379721</v>
+        <v>0.1375031246846421</v>
       </c>
       <c r="J23">
-        <v>0.007752243424404085</v>
+        <v>0.005396993969338132</v>
       </c>
       <c r="K23">
-        <v>-0.4059009629105702</v>
+        <v>-0.3844796819927853</v>
       </c>
       <c r="L23">
-        <v>-0.6808653523379501</v>
+        <v>-0.660343584330276</v>
       </c>
       <c r="M23">
-        <v>-0.6290055510176999</v>
+        <v>-0.6127355638936063</v>
       </c>
       <c r="N23">
-        <v>-0.5826112935258686</v>
+        <v>-0.5631256427215817</v>
       </c>
       <c r="O23">
-        <v>-0.4980215224411933</v>
+        <v>-0.4774900201554068</v>
       </c>
       <c r="P23">
-        <v>-0.4059009629105702</v>
+        <v>-0.3844796819927853</v>
       </c>
       <c r="Q23">
-        <v>-0.3120138456327275</v>
+        <v>-0.2959074369696905</v>
       </c>
       <c r="R23">
-        <v>-0.2362582856643825</v>
+        <v>-0.2133831762162299</v>
       </c>
       <c r="S23">
-        <v>-0.1875672023811518</v>
+        <v>-0.1617123972455172</v>
       </c>
       <c r="T23">
-        <v>-0.13768853671991</v>
+        <v>-0.1103279673395892</v>
       </c>
     </row>
     <row r="24">
@@ -14001,43 +14001,43 @@
         </is>
       </c>
       <c r="H24">
-        <v>-0.1889578831058645</v>
+        <v>-0.1831147261014914</v>
       </c>
       <c r="I24">
-        <v>0.1327116504290296</v>
+        <v>0.1350369720875784</v>
       </c>
       <c r="J24">
-        <v>0.004988553944890132</v>
+        <v>0.003915876801680832</v>
       </c>
       <c r="K24">
-        <v>-0.1854118738502842</v>
+        <v>-0.1785893086645667</v>
       </c>
       <c r="L24">
-        <v>-0.4602265954673859</v>
+        <v>-0.4649684790586853</v>
       </c>
       <c r="M24">
-        <v>-0.4109149079112364</v>
+        <v>-0.4154883456029336</v>
       </c>
       <c r="N24">
-        <v>-0.3562558322924651</v>
+        <v>-0.358318296277535</v>
       </c>
       <c r="O24">
-        <v>-0.2767524515129072</v>
+        <v>-0.2698399395404846</v>
       </c>
       <c r="P24">
-        <v>-0.1854118738502842</v>
+        <v>-0.1785893086645667</v>
       </c>
       <c r="Q24">
-        <v>-0.09630601969289393</v>
+        <v>-0.09008199488237223</v>
       </c>
       <c r="R24">
-        <v>-0.02334182334123727</v>
+        <v>-0.01445770825028103</v>
       </c>
       <c r="S24">
-        <v>0.02185289638685428</v>
+        <v>0.03175994551138536</v>
       </c>
       <c r="T24">
-        <v>0.0567593032052706</v>
+        <v>0.06508679198580132</v>
       </c>
     </row>
     <row r="25">
@@ -14071,43 +14071,43 @@
         </is>
       </c>
       <c r="H25">
-        <v>0.4928832352681846</v>
+        <v>0.5216747421585012</v>
       </c>
       <c r="I25">
-        <v>0.2081492105235483</v>
+        <v>0.1656690180157772</v>
       </c>
       <c r="J25">
-        <v>0.142336995204372</v>
+        <v>0.06199340762075325</v>
       </c>
       <c r="K25">
-        <v>0.4948766498617353</v>
+        <v>0.4970093760277954</v>
       </c>
       <c r="L25">
-        <v>0.194505971157467</v>
+        <v>0.2544938193727065</v>
       </c>
       <c r="M25">
-        <v>0.214159402191094</v>
+        <v>0.2818463068147971</v>
       </c>
       <c r="N25">
-        <v>0.2338548175674627</v>
+        <v>0.3183431310005265</v>
       </c>
       <c r="O25">
-        <v>0.3454576614088294</v>
+        <v>0.4034339590777929</v>
       </c>
       <c r="P25">
-        <v>0.4948766498617353</v>
+        <v>0.4970093760277954</v>
       </c>
       <c r="Q25">
-        <v>0.5778643295666729</v>
+        <v>0.621124205496744</v>
       </c>
       <c r="R25">
-        <v>0.7787218439451356</v>
+        <v>0.7744348303172901</v>
       </c>
       <c r="S25">
-        <v>0.9380251412749596</v>
+        <v>0.8405695748132813</v>
       </c>
       <c r="T25">
-        <v>1.018700735436573</v>
+        <v>0.867919380982383</v>
       </c>
     </row>
   </sheetData>

</xml_diff>